<commit_message>
fix: steal/lockpick/butcher/stealth/barter 的 mode 改成 passive，不該被拖進 ability slot
這 5 個技能都不是靠拖進 hotbar 主動施放的：steal/lockpick/butcher 是透過 findAb(id)
在 com_lock.js/com_stolen.js/com_loot.js 當作「有沒有學會」的權限判斷(互動選項開關)；
stealth/barter 完全還沒接程式碼，barter 描述本身就是「交易時自動套用」的被動效果。

原本標成 active 是錯的——AbilityItem.leftButtonDown()(uiclass.js)本來就是靠
mode!==GM.PASSIVE 才允許拖曳(DragService.onAbilityDown)，這5個從設計意圖上就
不該能被拖進 slot。
</commit_message>
<xml_diff>
--- a/xls/ability.xlsx
+++ b/xls/ability.xlsx
@@ -56,7 +56,7 @@
     <t>🧤</t>
   </si>
   <si>
-    <t>active</t>
+    <t>passive</t>
   </si>
   <si>
     <t xml:space="preserve">"lab":"偷竊",
@@ -132,6 +132,9 @@
     <t>🗡️</t>
   </si>
   <si>
+    <t>active</t>
+  </si>
+  <si>
     <t>atk</t>
   </si>
   <si>
@@ -184,9 +187,6 @@
   </si>
   <si>
     <t>⚔️</t>
-  </si>
-  <si>
-    <t>passive</t>
   </si>
   <si>
     <t>buff</t>
@@ -1118,81 +1118,81 @@
         <v>32</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>50</v>
@@ -1217,7 +1217,7 @@
         <v>55</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>50</v>
@@ -1292,10 +1292,10 @@
         <v>61</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1" t="s">
@@ -1317,7 +1317,7 @@
         <v>66</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>50</v>
@@ -1342,7 +1342,7 @@
         <v>71</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>50</v>
@@ -1419,10 +1419,10 @@
         <v>77</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="2" t="s">
@@ -1444,10 +1444,10 @@
         <v>82</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>83</v>
@@ -1467,10 +1467,10 @@
         <v>87</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>88</v>
@@ -1493,10 +1493,10 @@
         <v>93</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>94</v>
@@ -1583,10 +1583,10 @@
         <v>99</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="2" t="s">
@@ -1608,10 +1608,10 @@
         <v>103</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>62</v>
@@ -1631,10 +1631,10 @@
         <v>107</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>108</v>
@@ -1657,10 +1657,10 @@
         <v>112</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>113</v>
@@ -1748,10 +1748,10 @@
         <v>117</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="2" t="s">
@@ -1773,10 +1773,10 @@
         <v>120</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>62</v>
@@ -1796,10 +1796,10 @@
         <v>123</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>124</v>
@@ -1893,7 +1893,7 @@
         <v>127</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>126</v>
@@ -1917,7 +1917,7 @@
         <v>132</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>126</v>
@@ -1940,7 +1940,7 @@
         <v>136</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>126</v>
@@ -1963,7 +1963,7 @@
         <v>140</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>126</v>
@@ -2053,7 +2053,7 @@
         <v>146</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>50</v>
@@ -2075,7 +2075,7 @@
         <v>150</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>50</v>
@@ -2095,7 +2095,7 @@
         <v>154</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>50</v>

</xml_diff>